<commit_message>
Updated definitions and new fish use score csv
</commit_message>
<xml_diff>
--- a/data/inputs/Original Excel/Fish Use Score calculator - Normalized.xlsx
+++ b/data/inputs/Original Excel/Fish Use Score calculator - Normalized.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lichenlandwater.sharepoint.com/Shared Documents/Projects/20240007_Atlas Process (GRMW)/07_GIS/Analysis/WebApp - Scoring/Data In/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lichenlandwater.sharepoint.com/Shared Documents/Projects/20240007_Atlas Process (GRMW)/04_Analysis/Fish Use Score Updates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="341" documentId="8_{A35F3C96-1814-4CC4-A2E6-1EFE3FC1917D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABF79D04-65B1-4A7B-9D2A-3332D44F4441}"/>
+  <xr:revisionPtr revIDLastSave="349" documentId="8_{A35F3C96-1814-4CC4-A2E6-1EFE3FC1917D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6961CF5-CB5B-4193-A939-418686D9648E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{C64114D2-1330-4B94-B05B-7575C36C9CAD}"/>
+    <workbookView xWindow="-23136" yWindow="-5880" windowWidth="23232" windowHeight="13872" firstSheet="1" activeTab="2" xr2:uid="{C64114D2-1330-4B94-B05B-7575C36C9CAD}"/>
   </bookViews>
   <sheets>
     <sheet name="Rank Comparison" sheetId="8" r:id="rId1"/>
@@ -23,8 +23,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">'Fish Use Scores - Normalized'!$D$2:$D$30</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'Fish Use Scores - Normalized'!$C$2:$C$30</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'Fish Use Scores - Normalized'!$E$2:$E$30</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'Fish Use Scores - Normalized'!$E$2:$E$30</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'Fish Use Scores - Normalized'!$C$2:$C$30</definedName>
     <definedName name="_xlchart.v1.3" hidden="1">'Fish Use Scores - Normalized'!$H$2:$H$30</definedName>
     <definedName name="_xlchart.v1.4" hidden="1">'Migration Score Calcs'!$E$1</definedName>
     <definedName name="_xlchart.v1.5" hidden="1">'Migration Score Calcs'!$E$2:$E$30</definedName>
@@ -1432,7 +1432,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.1</cx:f>
+        <cx:f>_xlchart.v1.2</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1495,7 +1495,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.2</cx:f>
+        <cx:f>_xlchart.v1.1</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -5098,7 +5098,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="8622030" y="6416040"/>
+              <a:off x="8317230" y="6416040"/>
               <a:ext cx="4575810" cy="2748915"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -6233,15 +6233,15 @@
       </c>
       <c r="H3" s="25">
         <f>'Fish Use Scores - Normalized'!F2</f>
-        <v>1.7222227578185711</v>
+        <v>1.8587228943187077</v>
       </c>
       <c r="I3" s="2">
         <f>RANK(H3,$H$3:$H$31)</f>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J3" s="2">
         <f>$G3-I3</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -6270,15 +6270,15 @@
       </c>
       <c r="H4" s="25">
         <f>'Fish Use Scores - Normalized'!F3</f>
-        <v>1.1597400849138049</v>
+        <v>1.2962402214139412</v>
       </c>
       <c r="I4" s="2">
         <f t="shared" ref="I4:I31" si="1">RANK(H4,$H$3:$H$31)</f>
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="J4" s="2">
         <f>$G4-I4</f>
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -6305,11 +6305,11 @@
       </c>
       <c r="H5" s="25">
         <f>'Fish Use Scores - Normalized'!F4</f>
-        <v>0.71249937410552067</v>
+        <v>0.7575444191505657</v>
       </c>
       <c r="I5" s="2">
         <f t="shared" si="1"/>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J5" s="61" t="s">
         <v>164</v>
@@ -6339,11 +6339,11 @@
       </c>
       <c r="H6" s="25">
         <f>'Fish Use Scores - Normalized'!F5</f>
-        <v>1.0476152360339706</v>
+        <v>1.0176602810790156</v>
       </c>
       <c r="I6" s="2">
         <f t="shared" si="1"/>
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J6" s="61" t="s">
         <v>164</v>
@@ -6375,15 +6375,15 @@
       </c>
       <c r="H7" s="25">
         <f>'Fish Use Scores - Normalized'!F6</f>
-        <v>1.9294642885662403</v>
+        <v>1.9136916977936493</v>
       </c>
       <c r="I7" s="2">
         <f t="shared" si="1"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J7" s="2">
         <f t="shared" ref="J7:J31" si="2">$G7-I7</f>
-        <v>-3</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -6412,7 +6412,7 @@
       </c>
       <c r="H8" s="25">
         <f>'Fish Use Scores - Normalized'!F7</f>
-        <v>2.6186654438246517</v>
+        <v>2.5278928530520606</v>
       </c>
       <c r="I8" s="2">
         <f t="shared" si="1"/>
@@ -6449,15 +6449,15 @@
       </c>
       <c r="H9" s="25">
         <f>'Fish Use Scores - Normalized'!F8</f>
-        <v>4.137684680046803</v>
+        <v>4.0469120892742119</v>
       </c>
       <c r="I9" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="2">
         <f t="shared" si="2"/>
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -6486,7 +6486,7 @@
       </c>
       <c r="H10" s="25">
         <f>'Fish Use Scores - Normalized'!F9</f>
-        <v>0.9249656154626883</v>
+        <v>0.89501066050773326</v>
       </c>
       <c r="I10" s="2">
         <f t="shared" si="1"/>
@@ -6523,7 +6523,7 @@
       </c>
       <c r="H11" s="25">
         <f>'Fish Use Scores - Normalized'!F10</f>
-        <v>3.747142519227749</v>
+        <v>3.686324883410113</v>
       </c>
       <c r="I11" s="2">
         <f t="shared" si="1"/>
@@ -6560,15 +6560,15 @@
       </c>
       <c r="H12" s="25">
         <f>'Fish Use Scores - Normalized'!F11</f>
-        <v>3.7656023580718143</v>
+        <v>2.6412974629451575</v>
       </c>
       <c r="I12" s="2">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J12" s="2">
         <f t="shared" si="2"/>
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -6597,15 +6597,15 @@
       </c>
       <c r="H13" s="25">
         <f>'Fish Use Scores - Normalized'!F12</f>
-        <v>0.79210416710998321</v>
+        <v>6.7903578662097193</v>
       </c>
       <c r="I13" s="2">
         <f t="shared" si="1"/>
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="J13" s="2">
         <f t="shared" si="2"/>
-        <v>-1</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -6634,15 +6634,15 @@
       </c>
       <c r="H14" s="25">
         <f>'Fish Use Scores - Normalized'!F13</f>
-        <v>2.700176272798247</v>
+        <v>1.6152765394085735</v>
       </c>
       <c r="I14" s="2">
         <f t="shared" si="1"/>
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="J14" s="2">
         <f t="shared" si="2"/>
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -6671,15 +6671,15 @@
       </c>
       <c r="H15" s="25">
         <f>'Fish Use Scores - Normalized'!F14</f>
-        <v>0.77511614563043574</v>
+        <v>0.77395158443445566</v>
       </c>
       <c r="I15" s="2">
         <f t="shared" si="1"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J15" s="2">
         <f t="shared" si="2"/>
-        <v>-4</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -6708,15 +6708,15 @@
       </c>
       <c r="H16" s="25">
         <f>'Fish Use Scores - Normalized'!F15</f>
-        <v>2.1732350252757144</v>
+        <v>1.0112825608475753</v>
       </c>
       <c r="I16" s="2">
         <f t="shared" si="1"/>
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="J16" s="2">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -6745,15 +6745,15 @@
       </c>
       <c r="H17" s="25">
         <f>'Fish Use Scores - Normalized'!F16</f>
-        <v>3.1625219467760632</v>
+        <v>2.5454730750658574</v>
       </c>
       <c r="I17" s="2">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J17" s="2">
         <f t="shared" si="2"/>
-        <v>-1</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -6782,15 +6782,15 @@
       </c>
       <c r="H18" s="25">
         <f>'Fish Use Scores - Normalized'!F17</f>
-        <v>1.3985227380784215</v>
+        <v>0.74598075473290948</v>
       </c>
       <c r="I18" s="2">
         <f t="shared" si="1"/>
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="J18" s="2">
         <f t="shared" si="2"/>
-        <v>-4</v>
+        <v>-15</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -6819,15 +6819,15 @@
       </c>
       <c r="H19" s="25">
         <f>'Fish Use Scores - Normalized'!F18</f>
-        <v>0</v>
+        <v>0.99385049856315222</v>
       </c>
       <c r="I19" s="2">
         <f t="shared" si="1"/>
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="J19" s="2">
         <f t="shared" si="2"/>
-        <v>-2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -6856,15 +6856,15 @@
       </c>
       <c r="H20" s="25">
         <f>'Fish Use Scores - Normalized'!F19</f>
-        <v>1.3192443273449914</v>
+        <v>0.73137479024064622</v>
       </c>
       <c r="I20" s="2">
         <f t="shared" si="1"/>
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J20" s="2">
         <f t="shared" si="2"/>
-        <v>-5</v>
+        <v>-15</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -6893,15 +6893,15 @@
       </c>
       <c r="H21" s="25">
         <f>'Fish Use Scores - Normalized'!F20</f>
-        <v>1.0512874248960302</v>
+        <v>1.9980076246441505</v>
       </c>
       <c r="I21" s="2">
         <f t="shared" si="1"/>
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="J21" s="2">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -6930,15 +6930,15 @@
       </c>
       <c r="H22" s="25">
         <f>'Fish Use Scores - Normalized'!F21</f>
-        <v>1.8652655502151418</v>
+        <v>1.0390481206739461</v>
       </c>
       <c r="I22" s="2">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="J22" s="2">
         <f t="shared" si="2"/>
-        <v>-10</v>
+        <v>-16</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -6967,15 +6967,15 @@
       </c>
       <c r="H23" s="25">
         <f>'Fish Use Scores - Normalized'!F22</f>
-        <v>0.94371050384556376</v>
+        <v>2.0626908043525951</v>
       </c>
       <c r="I23" s="2">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="J23" s="2">
         <f t="shared" si="2"/>
-        <v>-1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -7004,15 +7004,15 @@
       </c>
       <c r="H24" s="25">
         <f>'Fish Use Scores - Normalized'!F23</f>
-        <v>1.1715857343269143</v>
+        <v>1.3571450981683322</v>
       </c>
       <c r="I24" s="2">
         <f t="shared" si="1"/>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="J24" s="2">
         <f t="shared" si="2"/>
-        <v>-3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -7041,15 +7041,15 @@
       </c>
       <c r="H25" s="25">
         <f>'Fish Use Scores - Normalized'!F24</f>
-        <v>2.9817301996759751</v>
+        <v>3.2436493871502989</v>
       </c>
       <c r="I25" s="2">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J25" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -7078,15 +7078,15 @@
       </c>
       <c r="H26" s="25">
         <f>'Fish Use Scores - Normalized'!F25</f>
-        <v>2.5357011855226115</v>
+        <v>1.2009330936825346</v>
       </c>
       <c r="I26" s="2">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="J26" s="2">
         <f t="shared" si="2"/>
-        <v>-9</v>
+        <v>-18</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
@@ -7115,15 +7115,15 @@
       </c>
       <c r="H27" s="25">
         <f>'Fish Use Scores - Normalized'!F26</f>
-        <v>1.3532265689263612</v>
+        <v>1.4458128501322305</v>
       </c>
       <c r="I27" s="2">
         <f t="shared" si="1"/>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J27" s="2">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -7152,15 +7152,15 @@
       </c>
       <c r="H28" s="25">
         <f>'Fish Use Scores - Normalized'!F27</f>
-        <v>2.4996651202714042</v>
+        <v>1.4815954930620125</v>
       </c>
       <c r="I28" s="2">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J28" s="2">
         <f t="shared" si="2"/>
-        <v>-10</v>
+        <v>-14</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
@@ -7189,15 +7189,15 @@
       </c>
       <c r="H29" s="25">
         <f>'Fish Use Scores - Normalized'!F28</f>
-        <v>2.6942058385075915</v>
+        <v>3.0030923483458301</v>
       </c>
       <c r="I29" s="2">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J29" s="2">
         <f t="shared" si="2"/>
-        <v>-1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
@@ -7226,15 +7226,15 @@
       </c>
       <c r="H30" s="25">
         <f>'Fish Use Scores - Normalized'!F29</f>
-        <v>3.2184935373254606</v>
+        <v>2.7613798838951396</v>
       </c>
       <c r="I30" s="2">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J30" s="2">
         <f t="shared" si="2"/>
-        <v>-4</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7263,15 +7263,15 @@
       </c>
       <c r="H31" s="67">
         <f>'Fish Use Scores - Normalized'!F30</f>
-        <v>3.5986053554012685</v>
+        <v>2.7612533802297055</v>
       </c>
       <c r="I31" s="5">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J31" s="5">
         <f t="shared" si="2"/>
-        <v>-2</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
@@ -7563,7 +7563,7 @@
     <col min="1" max="1" width="8.28515625" customWidth="1"/>
     <col min="2" max="2" width="37.85546875" customWidth="1"/>
     <col min="3" max="5" width="11.28515625" customWidth="1"/>
-    <col min="6" max="6" width="19.85546875" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" customWidth="1"/>
     <col min="8" max="8" width="16.5703125" customWidth="1"/>
     <col min="10" max="10" width="20" customWidth="1"/>
     <col min="11" max="11" width="15.28515625" customWidth="1"/>
@@ -7605,15 +7605,15 @@
       </c>
       <c r="C2" s="25">
         <f>$L$5*'Normalized Score Calculator'!C3
-+$L$6*'Normalized Score Calculator'!E3
-+$L$7*'Normalized Score Calculator'!G3
++$L$7*'Normalized Score Calculator'!E3
++$L$6*'Normalized Score Calculator'!G3
 +$L$8*'Normalized Score Calculator'!I3</f>
-        <v>0.77365461953640158</v>
+        <v>0.91015475603653817</v>
       </c>
       <c r="D2" s="25">
         <f>$M$5*'Normalized Score Calculator'!K3
-+$M$6*'Normalized Score Calculator'!M3
-+$M$7*'Normalized Score Calculator'!O3
++$M$7*'Normalized Score Calculator'!M3
++$M$6*'Normalized Score Calculator'!O3
 +$M$8*'Normalized Score Calculator'!Q3</f>
         <v>0.57806122583977326</v>
       </c>
@@ -7624,15 +7624,15 @@
       </c>
       <c r="F2" s="50">
         <f>C2*$L$17+D2*$L$18+E2*$L$19</f>
-        <v>1.7222227578185711</v>
+        <v>1.8587228943187077</v>
       </c>
       <c r="G2">
         <f>RANK(F2,$F$2:$F$30)</f>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H2" s="25">
         <f>F2*(100/F$35)</f>
-        <v>41.622861358277554</v>
+        <v>27.372974016113531</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -7644,15 +7644,15 @@
       </c>
       <c r="C3" s="25">
         <f>$L$5*'Normalized Score Calculator'!C4
-+$L$6*'Normalized Score Calculator'!E4
-+$L$7*'Normalized Score Calculator'!G4
++$L$7*'Normalized Score Calculator'!E4
++$L$6*'Normalized Score Calculator'!G4
 +$L$8*'Normalized Score Calculator'!I4</f>
-        <v>0.45696460492253749</v>
+        <v>0.59346474142267391</v>
       </c>
       <c r="D3" s="25">
         <f>$M$5*'Normalized Score Calculator'!K4
-+$M$6*'Normalized Score Calculator'!M4
-+$M$7*'Normalized Score Calculator'!O4
++$M$7*'Normalized Score Calculator'!M4
++$M$6*'Normalized Score Calculator'!O4
 +$M$8*'Normalized Score Calculator'!Q4</f>
         <v>0.33226856754887096</v>
       </c>
@@ -7663,15 +7663,15 @@
       </c>
       <c r="F3" s="50">
         <f>C3*$L$17+D3*$L$18+E3*$L$19</f>
-        <v>1.1597400849138049</v>
+        <v>1.2962402214139412</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G30" si="0">RANK(F3,$F$2:$F$30)</f>
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H3" s="25">
         <f t="shared" ref="H3:H30" si="1">F3*(100/F$35)</f>
-        <v>28.028720760342875</v>
+        <v>19.089424253533252</v>
       </c>
       <c r="K3" s="12" t="s">
         <v>7</v>
@@ -7691,15 +7691,15 @@
       </c>
       <c r="C4" s="25">
         <f>$L$5*'Normalized Score Calculator'!C5
-+$L$6*'Normalized Score Calculator'!E5
-+$L$7*'Normalized Score Calculator'!G5
++$L$7*'Normalized Score Calculator'!E5
++$L$6*'Normalized Score Calculator'!G5
 +$L$8*'Normalized Score Calculator'!I5</f>
-        <v>0.12355174559197681</v>
+        <v>0.16859679063702185</v>
       </c>
       <c r="D4" s="25">
         <f>$M$5*'Normalized Score Calculator'!K5
-+$M$6*'Normalized Score Calculator'!M5
-+$M$7*'Normalized Score Calculator'!O5
++$M$7*'Normalized Score Calculator'!M5
++$M$6*'Normalized Score Calculator'!O5
 +$M$8*'Normalized Score Calculator'!Q5</f>
         <v>0.58894762851354387</v>
       </c>
@@ -7710,15 +7710,15 @@
       </c>
       <c r="F4" s="50">
         <f t="shared" ref="F4:F30" si="2">C4*$L$17+D4*$L$18+E4*$L$19</f>
-        <v>0.71249937410552067</v>
+        <v>0.7575444191505657</v>
       </c>
       <c r="G4">
         <f t="shared" si="0"/>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H4" s="25">
         <f t="shared" si="1"/>
-        <v>17.219760063917228</v>
+        <v>11.156178128994785</v>
       </c>
       <c r="J4" s="10" t="s">
         <v>167</v>
@@ -7751,15 +7751,15 @@
       </c>
       <c r="C5" s="25">
         <f>$L$5*'Normalized Score Calculator'!C6
-+$L$6*'Normalized Score Calculator'!E6
-+$L$7*'Normalized Score Calculator'!G6
++$L$7*'Normalized Score Calculator'!E6
++$L$6*'Normalized Score Calculator'!G6
 +$L$8*'Normalized Score Calculator'!I6</f>
-        <v>0.30251498132843374</v>
+        <v>0.27256002637347876</v>
       </c>
       <c r="D5" s="25">
         <f>$M$5*'Normalized Score Calculator'!K6
-+$M$6*'Normalized Score Calculator'!M6
-+$M$7*'Normalized Score Calculator'!O6
++$M$7*'Normalized Score Calculator'!M6
++$M$6*'Normalized Score Calculator'!O6
 +$M$8*'Normalized Score Calculator'!Q6</f>
         <v>0.74510025470553687</v>
       </c>
@@ -7770,15 +7770,15 @@
       </c>
       <c r="F5" s="50">
         <f t="shared" si="2"/>
-        <v>1.0476152360339706</v>
+        <v>1.0176602810790156</v>
       </c>
       <c r="G5">
         <f t="shared" si="0"/>
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H5" s="25">
         <f t="shared" si="1"/>
-        <v>25.318875580004818</v>
+        <v>14.986843125648972</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="9" t="s">
@@ -7812,15 +7812,15 @@
       </c>
       <c r="C6" s="25">
         <f>$L$5*'Normalized Score Calculator'!C7
-+$L$6*'Normalized Score Calculator'!E7
-+$L$7*'Normalized Score Calculator'!G7
++$L$7*'Normalized Score Calculator'!E7
++$L$6*'Normalized Score Calculator'!G7
 +$L$8*'Normalized Score Calculator'!I7</f>
-        <v>0.92543662207829192</v>
+        <v>0.90966403130570106</v>
       </c>
       <c r="D6" s="25">
         <f>$M$5*'Normalized Score Calculator'!K7
-+$M$6*'Normalized Score Calculator'!M7
-+$M$7*'Normalized Score Calculator'!O7
++$M$7*'Normalized Score Calculator'!M7
++$M$6*'Normalized Score Calculator'!O7
 +$M$8*'Normalized Score Calculator'!Q7</f>
         <v>0.63352075404555208</v>
       </c>
@@ -7831,15 +7831,15 @@
       </c>
       <c r="F6" s="50">
         <f t="shared" si="2"/>
-        <v>1.9294642885662403</v>
+        <v>1.9136916977936493</v>
       </c>
       <c r="G6">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H6" s="25">
         <f t="shared" si="1"/>
-        <v>46.631496543724431</v>
+        <v>28.182486630293678</v>
       </c>
       <c r="J6" s="6" t="s">
         <v>165</v>
@@ -7872,15 +7872,15 @@
       </c>
       <c r="C7" s="25">
         <f>$L$5*'Normalized Score Calculator'!C8
-+$L$6*'Normalized Score Calculator'!E8
-+$L$7*'Normalized Score Calculator'!G8
++$L$7*'Normalized Score Calculator'!E8
++$L$6*'Normalized Score Calculator'!G8
 +$L$8*'Normalized Score Calculator'!I8</f>
-        <v>1.2599892945036624</v>
+        <v>1.1692167037310717</v>
       </c>
       <c r="D7" s="25">
         <f>$M$5*'Normalized Score Calculator'!K8
-+$M$6*'Normalized Score Calculator'!M8
-+$M$7*'Normalized Score Calculator'!O8
++$M$7*'Normalized Score Calculator'!M8
++$M$6*'Normalized Score Calculator'!O8
 +$M$8*'Normalized Score Calculator'!Q8</f>
         <v>0.80568075761591984</v>
       </c>
@@ -7891,7 +7891,7 @@
       </c>
       <c r="F7" s="50">
         <f t="shared" si="2"/>
-        <v>2.6186654438246517</v>
+        <v>2.5278928530520606</v>
       </c>
       <c r="G7">
         <f t="shared" si="0"/>
@@ -7899,7 +7899,7 @@
       </c>
       <c r="H7" s="25">
         <f t="shared" si="1"/>
-        <v>63.288182795868124</v>
+        <v>37.227682293909702</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>165</v>
@@ -7924,15 +7924,15 @@
       </c>
       <c r="C8" s="25">
         <f>$L$5*'Normalized Score Calculator'!C9
-+$L$6*'Normalized Score Calculator'!E9
-+$L$7*'Normalized Score Calculator'!G9
++$L$7*'Normalized Score Calculator'!E9
++$L$6*'Normalized Score Calculator'!G9
 +$L$8*'Normalized Score Calculator'!I9</f>
-        <v>1.1907151103197424</v>
+        <v>1.0999425195471517</v>
       </c>
       <c r="D8" s="25">
         <f>$M$5*'Normalized Score Calculator'!K9
-+$M$6*'Normalized Score Calculator'!M9
-+$M$7*'Normalized Score Calculator'!O9
++$M$7*'Normalized Score Calculator'!M9
++$M$6*'Normalized Score Calculator'!O9
 +$M$8*'Normalized Score Calculator'!Q9</f>
         <v>0.94966280077648235</v>
       </c>
@@ -7942,16 +7942,16 @@
         <v>1.9973067689505781</v>
       </c>
       <c r="F8" s="50">
-        <f>C8*$L$17+D8*$L$18+E8*$L$19</f>
-        <v>4.137684680046803</v>
+        <f t="shared" si="2"/>
+        <v>4.0469120892742119</v>
       </c>
       <c r="G8">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H8" s="25">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>59.597920595798293</v>
       </c>
       <c r="J8" s="7" t="s">
         <v>165</v>
@@ -7976,15 +7976,15 @@
       </c>
       <c r="C9" s="25">
         <f>$L$5*'Normalized Score Calculator'!C10
-+$L$6*'Normalized Score Calculator'!E10
-+$L$7*'Normalized Score Calculator'!G10
++$L$7*'Normalized Score Calculator'!E10
++$L$6*'Normalized Score Calculator'!G10
 +$L$8*'Normalized Score Calculator'!I10</f>
-        <v>0.26799975082449379</v>
+        <v>0.23804479586953881</v>
       </c>
       <c r="D9" s="25">
         <f>$M$5*'Normalized Score Calculator'!K10
-+$M$6*'Normalized Score Calculator'!M10
-+$M$7*'Normalized Score Calculator'!O10
++$M$7*'Normalized Score Calculator'!M10
++$M$6*'Normalized Score Calculator'!O10
 +$M$8*'Normalized Score Calculator'!Q10</f>
         <v>0.65696586463819451</v>
       </c>
@@ -7995,7 +7995,7 @@
       </c>
       <c r="F9" s="50">
         <f t="shared" si="2"/>
-        <v>0.9249656154626883</v>
+        <v>0.89501066050773326</v>
       </c>
       <c r="G9">
         <f t="shared" si="0"/>
@@ -8003,7 +8003,7 @@
       </c>
       <c r="H9" s="25">
         <f t="shared" si="1"/>
-        <v>22.354666606741663</v>
+        <v>13.180611068549107</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="9" t="s">
@@ -8029,15 +8029,15 @@
       </c>
       <c r="C10" s="25">
         <f>$L$5*'Normalized Score Calculator'!C11
-+$L$6*'Normalized Score Calculator'!E11
-+$L$7*'Normalized Score Calculator'!G11
++$L$7*'Normalized Score Calculator'!E11
++$L$6*'Normalized Score Calculator'!G11
 +$L$8*'Normalized Score Calculator'!I11</f>
-        <v>0.69917327089445869</v>
+        <v>0.6383556350768228</v>
       </c>
       <c r="D10" s="25">
         <f>$M$5*'Normalized Score Calculator'!K11
-+$M$6*'Normalized Score Calculator'!M11
-+$M$7*'Normalized Score Calculator'!O11
++$M$7*'Normalized Score Calculator'!M11
++$M$6*'Normalized Score Calculator'!O11
 +$M$8*'Normalized Score Calculator'!Q11</f>
         <v>0.70979214631612608</v>
       </c>
@@ -8048,15 +8048,15 @@
       </c>
       <c r="F10" s="50">
         <f t="shared" si="2"/>
-        <v>3.747142519227749</v>
+        <v>3.686324883410113</v>
       </c>
       <c r="G10">
-        <f>RANK(F10,$F$2:$F$30)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="H10" s="25">
         <f t="shared" si="1"/>
-        <v>90.561335843149934</v>
+        <v>54.287637795263457</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>166</v>
@@ -8080,18 +8080,18 @@
         <v>77</v>
       </c>
       <c r="C11" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C19
-+$L$6*'Normalized Score Calculator'!E19
-+$L$7*'Normalized Score Calculator'!G19
-+$L$8*'Normalized Score Calculator'!I19</f>
-        <v>1.1243030606193569</v>
+        <f>$L$9*'Normalized Score Calculator'!C12
++$L$11*'Normalized Score Calculator'!E12
++$L$10*'Normalized Score Calculator'!G12
++$L$12*'Normalized Score Calculator'!I12</f>
+        <v>0</v>
       </c>
       <c r="D11" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K19
-+$M$6*'Normalized Score Calculator'!M19
-+$M$7*'Normalized Score Calculator'!O19
-+$M$8*'Normalized Score Calculator'!Q19</f>
-        <v>0.7153733715265318</v>
+        <f>$M$9*'Normalized Score Calculator'!K19
++$M$11*'Normalized Score Calculator'!M19
++$M$10*'Normalized Score Calculator'!O19
++$M$12*'Normalized Score Calculator'!Q19</f>
+        <v>0.71537153701923184</v>
       </c>
       <c r="E11" s="25">
         <f>$P$5*'Normalized Score Calculator'!S19
@@ -8099,16 +8099,16 @@
         <v>1.9259259259259256</v>
       </c>
       <c r="F11" s="50">
-        <f>C11*$L$17+D11*$L$18+E11*$L$19</f>
-        <v>3.7656023580718143</v>
+        <f t="shared" si="2"/>
+        <v>2.6412974629451575</v>
       </c>
       <c r="G11">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H11" s="25">
         <f t="shared" si="1"/>
-        <v>91.007475176412427</v>
+        <v>38.89776525753998</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>166</v>
@@ -8132,18 +8132,18 @@
         <v>78</v>
       </c>
       <c r="C12" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C20
-+$L$6*'Normalized Score Calculator'!E20
-+$L$7*'Normalized Score Calculator'!G20
-+$L$8*'Normalized Score Calculator'!I20</f>
-        <v>1.7443443449164239E-3</v>
+        <f>$L$9*'Normalized Score Calculator'!C13
++$L$11*'Normalized Score Calculator'!E13
++$L$10*'Normalized Score Calculator'!G13
++$L$12*'Normalized Score Calculator'!I13</f>
+        <v>6</v>
       </c>
       <c r="D12" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K20
-+$M$6*'Normalized Score Calculator'!M20
-+$M$7*'Normalized Score Calculator'!O20
-+$M$8*'Normalized Score Calculator'!Q20</f>
-        <v>0.79035982276506678</v>
+        <f>$M$9*'Normalized Score Calculator'!K20
++$M$11*'Normalized Score Calculator'!M20
++$M$10*'Normalized Score Calculator'!O20
++$M$12*'Normalized Score Calculator'!Q20</f>
+        <v>0.79035786620971882</v>
       </c>
       <c r="E12" s="25">
         <f>$P$5*'Normalized Score Calculator'!S20
@@ -8152,15 +8152,15 @@
       </c>
       <c r="F12" s="50">
         <f t="shared" si="2"/>
-        <v>0.79210416710998321</v>
+        <v>6.7903578662097193</v>
       </c>
       <c r="G12">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="H12" s="25">
         <f t="shared" si="1"/>
-        <v>19.14365710199607</v>
+        <v>100</v>
       </c>
       <c r="J12" s="7" t="s">
         <v>166</v>
@@ -8184,18 +8184,18 @@
         <v>79</v>
       </c>
       <c r="C13" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C21
-+$L$6*'Normalized Score Calculator'!E21
-+$L$7*'Normalized Score Calculator'!G21
-+$L$8*'Normalized Score Calculator'!I21</f>
-        <v>1.084871040914142</v>
+        <f>$L$9*'Normalized Score Calculator'!C14
++$L$11*'Normalized Score Calculator'!E14
++$L$10*'Normalized Score Calculator'!G14
++$L$12*'Normalized Score Calculator'!I14</f>
+        <v>0</v>
       </c>
       <c r="D13" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K21
-+$M$6*'Normalized Score Calculator'!M21
-+$M$7*'Normalized Score Calculator'!O21
-+$M$8*'Normalized Score Calculator'!Q21</f>
-        <v>1.0227126392915122</v>
+        <f>$M$9*'Normalized Score Calculator'!K21
++$M$11*'Normalized Score Calculator'!M21
++$M$10*'Normalized Score Calculator'!O21
++$M$12*'Normalized Score Calculator'!Q21</f>
+        <v>1.0226839468159812</v>
       </c>
       <c r="E13" s="25">
         <f>$P$5*'Normalized Score Calculator'!S21
@@ -8204,15 +8204,15 @@
       </c>
       <c r="F13" s="50">
         <f t="shared" si="2"/>
-        <v>2.700176272798247</v>
+        <v>1.6152765394085735</v>
       </c>
       <c r="G13">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="H13" s="25">
         <f t="shared" si="1"/>
-        <v>65.258145112394217</v>
+        <v>23.787796920785823</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
@@ -8223,18 +8223,18 @@
         <v>80</v>
       </c>
       <c r="C14" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C22
-+$L$6*'Normalized Score Calculator'!E22
-+$L$7*'Normalized Score Calculator'!G22
-+$L$8*'Normalized Score Calculator'!I22</f>
-        <v>1.1631985035004016E-3</v>
+        <f>$L$9*'Normalized Score Calculator'!C15
++$L$11*'Normalized Score Calculator'!E15
++$L$10*'Normalized Score Calculator'!G15
++$L$12*'Normalized Score Calculator'!I15</f>
+        <v>0</v>
       </c>
       <c r="D14" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K22
-+$M$6*'Normalized Score Calculator'!M22
-+$M$7*'Normalized Score Calculator'!O22
-+$M$8*'Normalized Score Calculator'!Q22</f>
-        <v>0.7739529471269353</v>
+        <f>$M$9*'Normalized Score Calculator'!K22
++$M$11*'Normalized Score Calculator'!M22
++$M$10*'Normalized Score Calculator'!O22
++$M$12*'Normalized Score Calculator'!Q22</f>
+        <v>0.77395158443445566</v>
       </c>
       <c r="E14" s="25">
         <f>$P$5*'Normalized Score Calculator'!S22
@@ -8243,15 +8243,15 @@
       </c>
       <c r="F14" s="50">
         <f t="shared" si="2"/>
-        <v>0.77511614563043574</v>
+        <v>0.77395158443445566</v>
       </c>
       <c r="G14">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H14" s="25">
         <f t="shared" si="1"/>
-        <v>18.73308880612111</v>
+        <v>11.397802585424918</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -8262,18 +8262,18 @@
         <v>81</v>
       </c>
       <c r="C15" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C23
-+$L$6*'Normalized Score Calculator'!E23
-+$L$7*'Normalized Score Calculator'!G23
-+$L$8*'Normalized Score Calculator'!I23</f>
-        <v>1.1619282003848936</v>
+        <f>$L$9*'Normalized Score Calculator'!C16
++$L$11*'Normalized Score Calculator'!E16
++$L$10*'Normalized Score Calculator'!G16
++$L$12*'Normalized Score Calculator'!I16</f>
+        <v>0</v>
       </c>
       <c r="D15" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K23
-+$M$6*'Normalized Score Calculator'!M23
-+$M$7*'Normalized Score Calculator'!O23
-+$M$8*'Normalized Score Calculator'!Q23</f>
-        <v>0.81575126933526509</v>
+        <f>$M$9*'Normalized Score Calculator'!K23
++$M$11*'Normalized Score Calculator'!M23
++$M$10*'Normalized Score Calculator'!O23
++$M$12*'Normalized Score Calculator'!Q23</f>
+        <v>0.81572700529201969</v>
       </c>
       <c r="E15" s="25">
         <f>$P$5*'Normalized Score Calculator'!S23
@@ -8282,15 +8282,15 @@
       </c>
       <c r="F15" s="50">
         <f t="shared" si="2"/>
-        <v>2.1732350252757144</v>
+        <v>1.0112825608475753</v>
       </c>
       <c r="G15">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="H15" s="25">
         <f t="shared" si="1"/>
-        <v>52.522973433807721</v>
+        <v>14.892919942849179</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -8301,18 +8301,18 @@
         <v>82</v>
       </c>
       <c r="C16" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C24
-+$L$6*'Normalized Score Calculator'!E24
-+$L$7*'Normalized Score Calculator'!G24
-+$L$8*'Normalized Score Calculator'!I24</f>
-        <v>0.61704601945887039</v>
+        <f>$L$9*'Normalized Score Calculator'!C17
++$L$11*'Normalized Score Calculator'!E17
++$L$10*'Normalized Score Calculator'!G17
++$L$12*'Normalized Score Calculator'!I17</f>
+        <v>0</v>
       </c>
       <c r="D16" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K24
-+$M$6*'Normalized Score Calculator'!M24
-+$M$7*'Normalized Score Calculator'!O24
-+$M$8*'Normalized Score Calculator'!Q24</f>
-        <v>0.81510555694682285</v>
+        <f>$M$9*'Normalized Score Calculator'!K24
++$M$11*'Normalized Score Calculator'!M24
++$M$10*'Normalized Score Calculator'!O24
++$M$12*'Normalized Score Calculator'!Q24</f>
+        <v>0.81510270469548718</v>
       </c>
       <c r="E16" s="25">
         <f>$P$5*'Normalized Score Calculator'!S24
@@ -8321,15 +8321,15 @@
       </c>
       <c r="F16" s="50">
         <f t="shared" si="2"/>
-        <v>3.1625219467760632</v>
+        <v>2.5454730750658574</v>
       </c>
       <c r="G16">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H16" s="25">
         <f t="shared" si="1"/>
-        <v>76.432164152737968</v>
+        <v>37.486582080344817</v>
       </c>
       <c r="K16" s="12" t="s">
         <v>10</v>
@@ -8345,18 +8345,18 @@
         <v>83</v>
       </c>
       <c r="C17" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C25
-+$L$6*'Normalized Score Calculator'!E25
-+$L$7*'Normalized Score Calculator'!G25
-+$L$8*'Normalized Score Calculator'!I25</f>
-        <v>0.65252732250753365</v>
+        <f>$L$9*'Normalized Score Calculator'!C18
++$L$11*'Normalized Score Calculator'!E18
++$L$10*'Normalized Score Calculator'!G18
++$L$12*'Normalized Score Calculator'!I18</f>
+        <v>0</v>
       </c>
       <c r="D17" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K25
-+$M$6*'Normalized Score Calculator'!M25
-+$M$7*'Normalized Score Calculator'!O25
-+$M$8*'Normalized Score Calculator'!Q25</f>
-        <v>0.55043986001533241</v>
+        <f>$M$9*'Normalized Score Calculator'!K25
++$M$11*'Normalized Score Calculator'!M25
++$M$10*'Normalized Score Calculator'!O25
++$M$12*'Normalized Score Calculator'!Q25</f>
+        <v>0.55042519917735389</v>
       </c>
       <c r="E17" s="25">
         <f>$P$5*'Normalized Score Calculator'!S25
@@ -8365,15 +8365,15 @@
       </c>
       <c r="F17" s="50">
         <f t="shared" si="2"/>
-        <v>1.3985227380784215</v>
+        <v>0.74598075473290948</v>
       </c>
       <c r="G17">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H17" s="25">
         <f t="shared" si="1"/>
-        <v>33.799645120918257</v>
+        <v>10.985882768345245</v>
       </c>
       <c r="J17" s="2"/>
       <c r="K17" s="9" t="s">
@@ -8392,18 +8392,18 @@
         <v>84</v>
       </c>
       <c r="C18" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C26
-+$L$6*'Normalized Score Calculator'!E26
-+$L$7*'Normalized Score Calculator'!G26
-+$L$8*'Normalized Score Calculator'!I26</f>
-        <v>0</v>
+        <f>$L$9*'Normalized Score Calculator'!C19
++$L$11*'Normalized Score Calculator'!E19
++$L$10*'Normalized Score Calculator'!G19
++$L$12*'Normalized Score Calculator'!I19</f>
+        <v>0.99372984531154485</v>
       </c>
       <c r="D18" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K26
-+$M$6*'Normalized Score Calculator'!M26
-+$M$7*'Normalized Score Calculator'!O26
-+$M$8*'Normalized Score Calculator'!Q26</f>
-        <v>0</v>
+        <f>$M$9*'Normalized Score Calculator'!K26
++$M$11*'Normalized Score Calculator'!M26
++$M$10*'Normalized Score Calculator'!O26
++$M$12*'Normalized Score Calculator'!Q26</f>
+        <v>1.2065325160734291E-4</v>
       </c>
       <c r="E18" s="25">
         <f>$P$5*'Normalized Score Calculator'!S26
@@ -8412,15 +8412,15 @@
       </c>
       <c r="F18" s="50">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.99385049856315222</v>
       </c>
       <c r="G18">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="H18" s="25">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>14.636202069831487</v>
       </c>
       <c r="K18" s="6" t="s">
         <v>6</v>
@@ -8438,18 +8438,18 @@
         <v>85</v>
       </c>
       <c r="C19" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C27
-+$L$6*'Normalized Score Calculator'!E27
-+$L$7*'Normalized Score Calculator'!G27
-+$L$8*'Normalized Score Calculator'!I27</f>
-        <v>0.58981599895736747</v>
+        <f>$L$9*'Normalized Score Calculator'!C20
++$L$11*'Normalized Score Calculator'!E20
++$L$10*'Normalized Score Calculator'!G20
++$L$12*'Normalized Score Calculator'!I20</f>
+        <v>1.960523029119126E-3</v>
       </c>
       <c r="D19" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K27
-+$M$6*'Normalized Score Calculator'!M27
-+$M$7*'Normalized Score Calculator'!O27
-+$M$8*'Normalized Score Calculator'!Q27</f>
-        <v>0.53387277283206858</v>
+        <f>$M$9*'Normalized Score Calculator'!K27
++$M$11*'Normalized Score Calculator'!M27
++$M$10*'Normalized Score Calculator'!O27
++$M$12*'Normalized Score Calculator'!Q27</f>
+        <v>0.53385871165597154</v>
       </c>
       <c r="E19" s="25">
         <f>$P$5*'Normalized Score Calculator'!S27
@@ -8458,15 +8458,15 @@
       </c>
       <c r="F19" s="50">
         <f t="shared" si="2"/>
-        <v>1.3192443273449914</v>
+        <v>0.73137479024064622</v>
       </c>
       <c r="G19">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="H19" s="25">
         <f t="shared" si="1"/>
-        <v>31.883636124009065</v>
+        <v>10.770784171481218</v>
       </c>
       <c r="K19" s="7" t="s">
         <v>5</v>
@@ -8484,18 +8484,18 @@
         <v>86</v>
       </c>
       <c r="C20" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C28
-+$L$6*'Normalized Score Calculator'!E28
-+$L$7*'Normalized Score Calculator'!G28
-+$L$8*'Normalized Score Calculator'!I28</f>
-        <v>0.27259867471602917</v>
+        <f>$L$9*'Normalized Score Calculator'!C21
++$L$11*'Normalized Score Calculator'!E21
++$L$10*'Normalized Score Calculator'!G21
++$L$12*'Normalized Score Calculator'!I21</f>
+        <v>1.2193204085736402</v>
       </c>
       <c r="D20" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K28
-+$M$6*'Normalized Score Calculator'!M28
-+$M$7*'Normalized Score Calculator'!O28
-+$M$8*'Normalized Score Calculator'!Q28</f>
-        <v>0.77868875018000117</v>
+        <f>$M$9*'Normalized Score Calculator'!K28
++$M$11*'Normalized Score Calculator'!M28
++$M$10*'Normalized Score Calculator'!O28
++$M$12*'Normalized Score Calculator'!Q28</f>
+        <v>0.77868721607051028</v>
       </c>
       <c r="E20" s="25">
         <f>$P$5*'Normalized Score Calculator'!S28
@@ -8504,15 +8504,15 @@
       </c>
       <c r="F20" s="50">
         <f t="shared" si="2"/>
-        <v>1.0512874248960302</v>
+        <v>1.9980076246441505</v>
       </c>
       <c r="G20">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="H20" s="25">
         <f t="shared" si="1"/>
-        <v>25.407625427951622</v>
+        <v>29.424187414137126</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
@@ -8523,18 +8523,18 @@
         <v>87</v>
       </c>
       <c r="C21" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C29
-+$L$6*'Normalized Score Calculator'!E29
-+$L$7*'Normalized Score Calculator'!G29
-+$L$8*'Normalized Score Calculator'!I29</f>
-        <v>0.82751251105370627</v>
+        <f>$L$9*'Normalized Score Calculator'!C22
++$L$11*'Normalized Score Calculator'!E22
++$L$10*'Normalized Score Calculator'!G22
++$L$12*'Normalized Score Calculator'!I22</f>
+        <v>1.307355087426104E-3</v>
       </c>
       <c r="D21" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K29
-+$M$6*'Normalized Score Calculator'!M29
-+$M$7*'Normalized Score Calculator'!O29
-+$M$8*'Normalized Score Calculator'!Q29</f>
-        <v>0.6407160021243985</v>
+        <f>$M$9*'Normalized Score Calculator'!K29
++$M$11*'Normalized Score Calculator'!M29
++$M$10*'Normalized Score Calculator'!O29
++$M$12*'Normalized Score Calculator'!Q29</f>
+        <v>0.64070372854948299</v>
       </c>
       <c r="E21" s="25">
         <f>$P$5*'Normalized Score Calculator'!S29
@@ -8543,15 +8543,15 @@
       </c>
       <c r="F21" s="50">
         <f t="shared" si="2"/>
-        <v>1.8652655502151418</v>
+        <v>1.0390481206739461</v>
       </c>
       <c r="G21">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H21" s="25">
         <f t="shared" si="1"/>
-        <v>45.079934660319331</v>
+        <v>15.301816798853459</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
@@ -8562,18 +8562,18 @@
         <v>88</v>
       </c>
       <c r="C22" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C30
-+$L$6*'Normalized Score Calculator'!E30
-+$L$7*'Normalized Score Calculator'!G30
-+$L$8*'Normalized Score Calculator'!I30</f>
-        <v>0.27376213965653007</v>
+        <f>$L$9*'Normalized Score Calculator'!C23
++$L$11*'Normalized Score Calculator'!E23
++$L$10*'Normalized Score Calculator'!G23
++$L$12*'Normalized Score Calculator'!I23</f>
+        <v>1.3927453011784061</v>
       </c>
       <c r="D22" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K30
-+$M$6*'Normalized Score Calculator'!M30
-+$M$7*'Normalized Score Calculator'!O30
-+$M$8*'Normalized Score Calculator'!Q30</f>
-        <v>0.6699483641890337</v>
+        <f>$M$9*'Normalized Score Calculator'!K30
++$M$11*'Normalized Score Calculator'!M30
++$M$10*'Normalized Score Calculator'!O30
++$M$12*'Normalized Score Calculator'!Q30</f>
+        <v>0.66994550317418911</v>
       </c>
       <c r="E22" s="25">
         <f>$P$5*'Normalized Score Calculator'!S30
@@ -8582,15 +8582,15 @@
       </c>
       <c r="F22" s="50">
         <f t="shared" si="2"/>
-        <v>0.94371050384556376</v>
+        <v>2.0626908043525951</v>
       </c>
       <c r="G22">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H22" s="25">
         <f t="shared" si="1"/>
-        <v>22.807695047339593</v>
+        <v>30.37676135770381</v>
       </c>
     </row>
     <row r="23" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -8601,18 +8601,18 @@
         <v>89</v>
       </c>
       <c r="C23" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C31
-+$L$6*'Normalized Score Calculator'!E31
-+$L$7*'Normalized Score Calculator'!G31
-+$L$8*'Normalized Score Calculator'!I31</f>
-        <v>0.32902243095514805</v>
+        <f>$L$9*'Normalized Score Calculator'!C24
++$L$11*'Normalized Score Calculator'!E24
++$L$10*'Normalized Score Calculator'!G24
++$L$12*'Normalized Score Calculator'!I24</f>
+        <v>0.51458564090781789</v>
       </c>
       <c r="D23" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K31
-+$M$6*'Normalized Score Calculator'!M31
-+$M$7*'Normalized Score Calculator'!O31
-+$M$8*'Normalized Score Calculator'!Q31</f>
-        <v>0.84256330337176633</v>
+        <f>$M$9*'Normalized Score Calculator'!K31
++$M$11*'Normalized Score Calculator'!M31
++$M$10*'Normalized Score Calculator'!O31
++$M$12*'Normalized Score Calculator'!Q31</f>
+        <v>0.84255945726051418</v>
       </c>
       <c r="E23" s="25">
         <f>$P$5*'Normalized Score Calculator'!S31
@@ -8621,15 +8621,15 @@
       </c>
       <c r="F23" s="50">
         <f t="shared" si="2"/>
-        <v>1.1715857343269143</v>
+        <v>1.3571450981683322</v>
       </c>
       <c r="G23">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H23" s="25">
         <f t="shared" si="1"/>
-        <v>28.315007665438198</v>
+        <v>19.986356019934941</v>
       </c>
     </row>
     <row r="24" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -8640,18 +8640,18 @@
         <v>90</v>
       </c>
       <c r="C24" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C32
-+$L$6*'Normalized Score Calculator'!E32
-+$L$7*'Normalized Score Calculator'!G32
-+$L$8*'Normalized Score Calculator'!I32</f>
-        <v>0.558293547743413</v>
+        <f>$L$9*'Normalized Score Calculator'!C25
++$L$11*'Normalized Score Calculator'!E25
++$L$10*'Normalized Score Calculator'!G25
++$L$12*'Normalized Score Calculator'!I25</f>
+        <v>0.82021376229815501</v>
       </c>
       <c r="D24" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K32
-+$M$6*'Normalized Score Calculator'!M32
-+$M$7*'Normalized Score Calculator'!O32
-+$M$8*'Normalized Score Calculator'!Q32</f>
-        <v>0.69306628156219208</v>
+        <f>$M$9*'Normalized Score Calculator'!K32
++$M$11*'Normalized Score Calculator'!M32
++$M$10*'Normalized Score Calculator'!O32
++$M$12*'Normalized Score Calculator'!Q32</f>
+        <v>0.69306525448177358</v>
       </c>
       <c r="E24" s="25">
         <f>$P$5*'Normalized Score Calculator'!S32
@@ -8660,15 +8660,15 @@
       </c>
       <c r="F24" s="50">
         <f t="shared" si="2"/>
-        <v>2.9817301996759751</v>
+        <v>3.2436493871502989</v>
       </c>
       <c r="G24">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H24" s="25">
         <f t="shared" si="1"/>
-        <v>72.062770129749168</v>
+        <v>47.768460087963781</v>
       </c>
       <c r="K24" s="12" t="s">
         <v>7</v>
@@ -8683,18 +8683,18 @@
         <v>91</v>
       </c>
       <c r="C25" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C33
-+$L$6*'Normalized Score Calculator'!E33
-+$L$7*'Normalized Score Calculator'!G33
-+$L$8*'Normalized Score Calculator'!I33</f>
-        <v>1.3550314544618765</v>
+        <f>$L$9*'Normalized Score Calculator'!C26
++$L$11*'Normalized Score Calculator'!E26
++$L$10*'Normalized Score Calculator'!G26
++$L$12*'Normalized Score Calculator'!I26</f>
+        <v>2.0267355670452843E-2</v>
       </c>
       <c r="D25" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K33
-+$M$6*'Normalized Score Calculator'!M33
-+$M$7*'Normalized Score Calculator'!O33
-+$M$8*'Normalized Score Calculator'!Q33</f>
-        <v>0.58807713846814236</v>
+        <f>$M$9*'Normalized Score Calculator'!K33
++$M$11*'Normalized Score Calculator'!M33
++$M$10*'Normalized Score Calculator'!O33
++$M$12*'Normalized Score Calculator'!Q33</f>
+        <v>0.58807314541948941</v>
       </c>
       <c r="E25" s="25">
         <f>$P$5*'Normalized Score Calculator'!S33
@@ -8703,15 +8703,15 @@
       </c>
       <c r="F25" s="50">
         <f t="shared" si="2"/>
-        <v>2.5357011855226115</v>
+        <v>1.2009330936825346</v>
       </c>
       <c r="G25">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="H25" s="25">
         <f t="shared" si="1"/>
-        <v>61.283093845950802</v>
+        <v>17.6858586446325</v>
       </c>
       <c r="K25" s="10" t="s">
         <v>41</v>
@@ -8728,18 +8728,18 @@
         <v>92</v>
       </c>
       <c r="C26" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C34
-+$L$6*'Normalized Score Calculator'!E34
-+$L$7*'Normalized Score Calculator'!G34
-+$L$8*'Normalized Score Calculator'!I34</f>
-        <v>0.65714313180380912</v>
+        <f>$L$9*'Normalized Score Calculator'!C27
++$L$11*'Normalized Score Calculator'!E27
++$L$10*'Normalized Score Calculator'!G27
++$L$12*'Normalized Score Calculator'!I27</f>
+        <v>0.74973054929898542</v>
       </c>
       <c r="D26" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K34
-+$M$6*'Normalized Score Calculator'!M34
-+$M$7*'Normalized Score Calculator'!O34
-+$M$8*'Normalized Score Calculator'!Q34</f>
-        <v>0.69608343712255205</v>
+        <f>$M$9*'Normalized Score Calculator'!K34
++$M$11*'Normalized Score Calculator'!M34
++$M$10*'Normalized Score Calculator'!O34
++$M$12*'Normalized Score Calculator'!Q34</f>
+        <v>0.69608230083324496</v>
       </c>
       <c r="E26" s="25">
         <f>$P$5*'Normalized Score Calculator'!S34
@@ -8748,15 +8748,15 @@
       </c>
       <c r="F26" s="50">
         <f t="shared" si="2"/>
-        <v>1.3532265689263612</v>
+        <v>1.4458128501322305</v>
       </c>
       <c r="G26">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H26" s="25">
         <f t="shared" si="1"/>
-        <v>32.704922524716267</v>
+        <v>21.292145106621053</v>
       </c>
       <c r="J26" s="2"/>
       <c r="K26" s="9" t="s">
@@ -8774,18 +8774,18 @@
         <v>93</v>
       </c>
       <c r="C27" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C35
-+$L$6*'Normalized Score Calculator'!E35
-+$L$7*'Normalized Score Calculator'!G35
-+$L$8*'Normalized Score Calculator'!I35</f>
-        <v>1.2799920815500763</v>
+        <f>$L$9*'Normalized Score Calculator'!C28
++$L$11*'Normalized Score Calculator'!E28
++$L$10*'Normalized Score Calculator'!G28
++$L$12*'Normalized Score Calculator'!I28</f>
+        <v>0.26192470360552494</v>
       </c>
       <c r="D27" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K35
-+$M$6*'Normalized Score Calculator'!M35
-+$M$7*'Normalized Score Calculator'!O35
-+$M$8*'Normalized Score Calculator'!Q35</f>
-        <v>0.62708044612873548</v>
+        <f>$M$9*'Normalized Score Calculator'!K35
++$M$11*'Normalized Score Calculator'!M35
++$M$10*'Normalized Score Calculator'!O35
++$M$12*'Normalized Score Calculator'!Q35</f>
+        <v>0.62707819686389521</v>
       </c>
       <c r="E27" s="25">
         <f>$P$5*'Normalized Score Calculator'!S35
@@ -8794,15 +8794,15 @@
       </c>
       <c r="F27" s="50">
         <f t="shared" si="2"/>
-        <v>2.4996651202714042</v>
+        <v>1.4815954930620125</v>
       </c>
       <c r="G27">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="H27" s="25">
         <f t="shared" si="1"/>
-        <v>60.412170418049584</v>
+        <v>21.819107656089088</v>
       </c>
       <c r="K27" s="6" t="s">
         <v>39</v>
@@ -8819,18 +8819,18 @@
         <v>94</v>
       </c>
       <c r="C28" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C36
-+$L$6*'Normalized Score Calculator'!E36
-+$L$7*'Normalized Score Calculator'!G36
-+$L$8*'Normalized Score Calculator'!I36</f>
-        <v>0.6635408077110615</v>
+        <f>$L$9*'Normalized Score Calculator'!C29
++$L$11*'Normalized Score Calculator'!E29
++$L$10*'Normalized Score Calculator'!G29
++$L$12*'Normalized Score Calculator'!I29</f>
+        <v>0.97242762346231904</v>
       </c>
       <c r="D28" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K36
-+$M$6*'Normalized Score Calculator'!M36
-+$M$7*'Normalized Score Calculator'!O36
-+$M$8*'Normalized Score Calculator'!Q36</f>
-        <v>0.50177614190764164</v>
+        <f>$M$9*'Normalized Score Calculator'!K36
++$M$11*'Normalized Score Calculator'!M36
++$M$10*'Normalized Score Calculator'!O36
++$M$12*'Normalized Score Calculator'!Q36</f>
+        <v>0.50177583599462228</v>
       </c>
       <c r="E28" s="25">
         <f>$P$5*'Normalized Score Calculator'!S36
@@ -8839,15 +8839,15 @@
       </c>
       <c r="F28" s="50">
         <f t="shared" si="2"/>
-        <v>2.6942058385075915</v>
+        <v>3.0030923483458301</v>
       </c>
       <c r="G28">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H28" s="25">
         <f t="shared" si="1"/>
-        <v>65.113851026393732</v>
+        <v>44.225833269993963</v>
       </c>
       <c r="K28" s="6" t="s">
         <v>38</v>
@@ -8864,18 +8864,18 @@
         <v>95</v>
       </c>
       <c r="C29" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C37
-+$L$6*'Normalized Score Calculator'!E37
-+$L$7*'Normalized Score Calculator'!G37
-+$L$8*'Normalized Score Calculator'!I37</f>
-        <v>0.72034487238522216</v>
+        <f>$L$9*'Normalized Score Calculator'!C30
++$L$11*'Normalized Score Calculator'!E30
++$L$10*'Normalized Score Calculator'!G30
++$L$12*'Normalized Score Calculator'!I30</f>
+        <v>0.26323235814980817</v>
       </c>
       <c r="D29" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K37
-+$M$6*'Normalized Score Calculator'!M37
-+$M$7*'Normalized Score Calculator'!O37
-+$M$8*'Normalized Score Calculator'!Q37</f>
-        <v>0.76777829456986846</v>
+        <f>$M$9*'Normalized Score Calculator'!K37
++$M$11*'Normalized Score Calculator'!M37
++$M$10*'Normalized Score Calculator'!O37
++$M$12*'Normalized Score Calculator'!Q37</f>
+        <v>0.76777715537496138</v>
       </c>
       <c r="E29" s="25">
         <f>$P$5*'Normalized Score Calculator'!S37
@@ -8884,15 +8884,15 @@
       </c>
       <c r="F29" s="50">
         <f t="shared" si="2"/>
-        <v>3.2184935373254606</v>
+        <v>2.7613798838951396</v>
       </c>
       <c r="G29">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H29" s="25">
         <f t="shared" si="1"/>
-        <v>77.784891459855146</v>
+        <v>40.666190770833438</v>
       </c>
       <c r="K29" s="6" t="s">
         <v>37</v>
@@ -8909,18 +8909,18 @@
         <v>96</v>
       </c>
       <c r="C30" s="25">
-        <f>$L$5*'Normalized Score Calculator'!C38
-+$L$6*'Normalized Score Calculator'!E38
-+$L$7*'Normalized Score Calculator'!G38
-+$L$8*'Normalized Score Calculator'!I38</f>
-        <v>1.1626924956058775</v>
+        <f>$L$9*'Normalized Score Calculator'!C31
++$L$11*'Normalized Score Calculator'!E31
++$L$10*'Normalized Score Calculator'!G31
++$L$12*'Normalized Score Calculator'!I31</f>
+        <v>0.32534112354495875</v>
       </c>
       <c r="D30" s="25">
-        <f>$M$5*'Normalized Score Calculator'!K38
-+$M$6*'Normalized Score Calculator'!M38
-+$M$7*'Normalized Score Calculator'!O38
-+$M$8*'Normalized Score Calculator'!Q38</f>
-        <v>0.50998693386946525</v>
+        <f>$M$9*'Normalized Score Calculator'!K38
++$M$11*'Normalized Score Calculator'!M38
++$M$10*'Normalized Score Calculator'!O38
++$M$12*'Normalized Score Calculator'!Q38</f>
+        <v>0.50998633075882138</v>
       </c>
       <c r="E30" s="25">
         <f>$P$5*'Normalized Score Calculator'!S38
@@ -8929,15 +8929,15 @@
       </c>
       <c r="F30" s="50">
         <f t="shared" si="2"/>
-        <v>3.5986053554012685</v>
+        <v>2.7612533802297055</v>
       </c>
       <c r="G30">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H30" s="25">
         <f t="shared" si="1"/>
-        <v>86.971473992565407</v>
+        <v>40.664327781165937</v>
       </c>
       <c r="K30" s="24" t="s">
         <v>71</v>
@@ -8950,13 +8950,12 @@
       <c r="B31" s="93" t="s">
         <v>174</v>
       </c>
-      <c r="C31" s="91">
-        <f>SUM(C2:C30)</f>
-        <v>19.333333333333329</v>
+      <c r="C31" s="25">
+        <v>19.333333333333325</v>
       </c>
       <c r="D31" s="91">
         <f t="shared" ref="D31:E31" si="3">SUM(D2:D30)</f>
-        <v>19.333333333333336</v>
+        <v>19.333333333333325</v>
       </c>
       <c r="E31" s="91">
         <f t="shared" si="3"/>
@@ -8964,33 +8963,33 @@
       </c>
       <c r="F31" s="92">
         <f>SUM(F2:F30)</f>
-        <v>57.999999999999993</v>
+        <v>58.203453216784823</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B32" s="22"/>
       <c r="C32" s="45">
-        <f>C31/$F$31</f>
-        <v>0.33333333333333331</v>
+        <f t="shared" ref="C32:E32" si="4">C31/$F$31</f>
+        <v>0.33216814922173626</v>
       </c>
       <c r="D32" s="45">
-        <f t="shared" ref="D32:E32" si="4">D31/$F$31</f>
-        <v>0.33333333333333343</v>
+        <f t="shared" si="4"/>
+        <v>0.33216814922173626</v>
       </c>
       <c r="E32" s="45">
         <f t="shared" si="4"/>
-        <v>0.33333333333333331</v>
+        <v>0.33216814922173632</v>
       </c>
       <c r="F32" s="22"/>
     </row>
     <row r="35" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F35" s="50">
         <f>MAX(F2:F30)</f>
-        <v>4.137684680046803</v>
+        <v>6.7903578662097193</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:C30">
+  <conditionalFormatting sqref="C2:C32">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -10190,7 +10189,7 @@
       </c>
       <c r="I19" s="82">
         <f>H19/$H$40*$B$41</f>
-        <v>4.6076589784541842E-2</v>
+        <v>4.5871860991868935E-2</v>
       </c>
       <c r="J19" s="81">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A19, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10222,7 +10221,7 @@
       </c>
       <c r="Q19" s="82">
         <f>P19/$P$40*$B$41</f>
-        <v>0.2027305274121752</v>
+        <v>0.20272318938297548</v>
       </c>
       <c r="R19" s="81">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A19, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10243,7 +10242,7 @@
       <c r="V19" s="80"/>
       <c r="W19" s="25">
         <f t="shared" si="11"/>
-        <v>11.75863533250703</v>
+        <v>11.758423265685158</v>
       </c>
       <c r="X19" s="80">
         <f t="shared" ref="X19:X38" si="22">RANK(W19,$W$3:$W$38)</f>
@@ -10284,7 +10283,7 @@
       </c>
       <c r="I20" s="44">
         <f t="shared" ref="I20:I38" si="23">H20/$H$40*$B$41</f>
-        <v>5.7563363382241986E-3</v>
+        <v>5.7307596235789829E-3</v>
       </c>
       <c r="J20" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A20, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10316,7 +10315,7 @@
       </c>
       <c r="Q20" s="44">
         <f t="shared" ref="Q20:Q38" si="24">P20/$P$40*$B$41</f>
-        <v>0.21621799903298144</v>
+        <v>0.21621017281158966</v>
       </c>
       <c r="R20" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A20, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10336,7 +10335,7 @@
       </c>
       <c r="W20" s="25">
         <f t="shared" si="11"/>
-        <v>3.1671956273984914</v>
+        <v>3.1671622244624542</v>
       </c>
       <c r="X20">
         <f t="shared" si="22"/>
@@ -10377,7 +10376,7 @@
       </c>
       <c r="I21" s="44">
         <f t="shared" si="23"/>
-        <v>3.5800744350166687</v>
+        <v>3.5641673481383331</v>
       </c>
       <c r="J21" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A21, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10409,7 +10408,7 @@
       </c>
       <c r="Q21" s="44">
         <f t="shared" si="24"/>
-        <v>3.1707917964822885</v>
+        <v>3.1706770265801638</v>
       </c>
       <c r="R21" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A21, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10429,7 +10428,7 @@
       </c>
       <c r="W21" s="25">
         <f t="shared" si="11"/>
-        <v>9.1524064736641986</v>
+        <v>9.1363846168837384</v>
       </c>
       <c r="X21">
         <f t="shared" si="22"/>
@@ -10470,7 +10469,7 @@
       </c>
       <c r="I22" s="44">
         <f t="shared" si="23"/>
-        <v>3.8385550615513248E-3</v>
+        <v>3.8214994863224575E-3</v>
       </c>
       <c r="J22" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A22, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10502,7 +10501,7 @@
       </c>
       <c r="Q22" s="44">
         <f t="shared" si="24"/>
-        <v>0.15059049648045575</v>
+        <v>0.1505850457105373</v>
       </c>
       <c r="R22" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A22, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10522,7 +10521,7 @@
       </c>
       <c r="W22" s="25">
         <f t="shared" si="11"/>
-        <v>3.0996503435692926</v>
+        <v>3.099627837224145</v>
       </c>
       <c r="X22">
         <f t="shared" si="22"/>
@@ -10563,7 +10562,7 @@
       </c>
       <c r="I23" s="44">
         <f t="shared" si="23"/>
-        <v>3.2482962071620576</v>
+        <v>3.2338632865868591</v>
       </c>
       <c r="J23" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A23, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10595,7 +10594,7 @@
       </c>
       <c r="Q23" s="44">
         <f t="shared" si="24"/>
-        <v>2.6814078551188381</v>
+        <v>2.6813107989458564</v>
       </c>
       <c r="R23" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A23, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10615,7 +10614,7 @@
       </c>
       <c r="W23" s="25">
         <f t="shared" si="11"/>
-        <v>7.8374285364035661</v>
+        <v>7.8228985596553855</v>
       </c>
       <c r="X23">
         <f t="shared" si="22"/>
@@ -10656,7 +10655,7 @@
       </c>
       <c r="I24" s="44">
         <f t="shared" si="23"/>
-        <v>0.19964012543653456</v>
+        <v>0.19875307884648066</v>
       </c>
       <c r="J24" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A24, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10688,7 +10687,7 @@
       </c>
       <c r="Q24" s="44">
         <f t="shared" si="24"/>
-        <v>0.31520093576000585</v>
+        <v>0.31518952675466311</v>
       </c>
       <c r="R24" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A24, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10708,7 +10707,7 @@
       </c>
       <c r="W24" s="25">
         <f t="shared" si="11"/>
-        <v>8.8963822974932807</v>
+        <v>8.8954838418978852</v>
       </c>
       <c r="X24">
         <f t="shared" si="22"/>
@@ -10749,7 +10748,7 @@
       </c>
       <c r="I25" s="44">
         <f t="shared" si="23"/>
-        <v>1.5672733101667695</v>
+        <v>1.5603095575522787</v>
       </c>
       <c r="J25" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A25, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10781,7 +10780,7 @@
       </c>
       <c r="Q25" s="44">
         <f t="shared" si="24"/>
-        <v>1.6201622178391075</v>
+        <v>1.6201035744871934</v>
       </c>
       <c r="R25" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A25, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10801,7 +10800,7 @@
       </c>
       <c r="W25" s="25">
         <f t="shared" si="11"/>
-        <v>5.095160002128547</v>
+        <v>5.0881376061621424</v>
       </c>
       <c r="X25">
         <f t="shared" si="22"/>
@@ -10838,11 +10837,11 @@
       </c>
       <c r="H26" s="25">
         <f>'Migration Score Calcs'!E18</f>
-        <v>0</v>
+        <v>1.6621845683827744E-2</v>
       </c>
       <c r="I26" s="44">
-        <f>H26/$H$40*$B$41</f>
-        <v>0</v>
+        <f t="shared" si="23"/>
+        <v>5.9243039652092926E-2</v>
       </c>
       <c r="J26" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A26, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10870,11 +10869,11 @@
       </c>
       <c r="P26" s="25">
         <f>'Migration Score Calcs'!F18</f>
-        <v>0</v>
+        <v>1.5221134236744052E-4</v>
       </c>
       <c r="Q26" s="44">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>4.8261300642937164E-4</v>
       </c>
       <c r="R26" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A26, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10894,7 +10893,7 @@
       </c>
       <c r="W26" s="25">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>5.9725652658522296E-2</v>
       </c>
       <c r="X26">
         <f t="shared" si="22"/>
@@ -10935,7 +10934,7 @@
       </c>
       <c r="I27" s="44">
         <f t="shared" si="23"/>
-        <v>1.3603259424512213</v>
+        <v>1.3542817041700907</v>
       </c>
       <c r="J27" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A27, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10967,7 +10966,7 @@
       </c>
       <c r="Q27" s="44">
         <f t="shared" si="24"/>
-        <v>1.553893869106052</v>
+        <v>1.5538376244016641</v>
       </c>
       <c r="R27" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A27, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -10987,7 +10986,7 @@
       </c>
       <c r="W27" s="25">
         <f t="shared" si="11"/>
-        <v>4.8219442856799439</v>
+        <v>4.8158438026944248</v>
       </c>
       <c r="X27">
         <f t="shared" si="22"/>
@@ -11028,7 +11027,7 @@
       </c>
       <c r="I28" s="44">
         <f t="shared" si="23"/>
-        <v>1.9192929560756908E-3</v>
+        <v>1.910765099923133E-3</v>
       </c>
       <c r="J28" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A28, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11060,7 +11059,7 @@
       </c>
       <c r="Q28" s="44">
         <f t="shared" si="24"/>
-        <v>0.16953370869271894</v>
+        <v>0.16952757225475568</v>
       </c>
       <c r="R28" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A28, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11080,7 +11079,7 @@
       </c>
       <c r="W28" s="25">
         <f t="shared" si="11"/>
-        <v>4.0365425441903549</v>
+        <v>4.036527879896239</v>
       </c>
       <c r="X28">
         <f t="shared" si="22"/>
@@ -11121,7 +11120,7 @@
       </c>
       <c r="I29" s="44">
         <f t="shared" si="23"/>
-        <v>1.2470680987623191</v>
+        <v>1.2415270909005316</v>
       </c>
       <c r="J29" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A29, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11153,7 +11152,7 @@
       </c>
       <c r="Q29" s="44">
         <f t="shared" si="24"/>
-        <v>1.3563469144805</v>
+        <v>1.3562978201808382</v>
       </c>
       <c r="R29" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A29, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11173,7 +11172,7 @@
       </c>
       <c r="W29" s="25">
         <f t="shared" si="11"/>
-        <v>6.5596313133783388</v>
+        <v>6.5540412112168909</v>
       </c>
       <c r="X29">
         <f t="shared" si="22"/>
@@ -11214,7 +11213,7 @@
       </c>
       <c r="I30" s="44">
         <f t="shared" si="23"/>
-        <v>5.7587272597286535E-3</v>
+        <v>5.7331399216741267E-3</v>
       </c>
       <c r="J30" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A30, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11246,7 +11245,7 @@
       </c>
       <c r="Q30" s="44">
         <f t="shared" si="24"/>
-        <v>0.31616938695107116</v>
+        <v>0.31615794289169286</v>
       </c>
       <c r="R30" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A30, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11266,7 +11265,7 @@
       </c>
       <c r="W30" s="25">
         <f t="shared" si="11"/>
-        <v>3.6054204345301382</v>
+        <v>3.6053834031327052</v>
       </c>
       <c r="X30">
         <f t="shared" si="22"/>
@@ -11307,7 +11306,7 @@
       </c>
       <c r="I31" s="44">
         <f t="shared" si="23"/>
-        <v>0.18811768854516797</v>
+        <v>0.18728183876903737</v>
       </c>
       <c r="J31" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A31, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11339,7 +11338,7 @@
       </c>
       <c r="Q31" s="44">
         <f t="shared" si="24"/>
-        <v>0.42503192145977964</v>
+        <v>0.42501653701477132</v>
       </c>
       <c r="R31" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A31, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11359,7 +11358,7 @@
       </c>
       <c r="W31" s="25">
         <f t="shared" si="11"/>
-        <v>4.4782391525465073</v>
+        <v>4.4773879183253689</v>
       </c>
       <c r="X31">
         <f t="shared" si="22"/>
@@ -11400,7 +11399,7 @@
       </c>
       <c r="I32" s="44">
         <f t="shared" si="23"/>
-        <v>5.7569687755253769E-3</v>
+        <v>5.7313892508170537E-3</v>
       </c>
       <c r="J32" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A32, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11432,7 +11431,7 @@
       </c>
       <c r="Q32" s="44">
         <f t="shared" si="24"/>
-        <v>0.1135021675548164</v>
+        <v>0.11349805923314241</v>
       </c>
       <c r="R32" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A32, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11452,7 +11451,7 @@
       </c>
       <c r="W32" s="25">
         <f t="shared" si="11"/>
-        <v>8.214342039293749</v>
+        <v>8.2143123514473668</v>
       </c>
       <c r="X32">
         <f t="shared" si="22"/>
@@ -11484,7 +11483,7 @@
         <v>1</v>
       </c>
       <c r="G33" s="44">
-        <f>F33/$F$40*$B$41</f>
+        <f t="shared" si="16"/>
         <v>1.5378700499807765</v>
       </c>
       <c r="H33" s="25">
@@ -11493,7 +11492,7 @@
       </c>
       <c r="I33" s="44">
         <f t="shared" si="23"/>
-        <v>0.80748028946485617</v>
+        <v>0.80389247045432743</v>
       </c>
       <c r="J33" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A33, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11525,7 +11524,7 @@
       </c>
       <c r="Q33" s="44">
         <f t="shared" si="24"/>
-        <v>0.44126990359890333</v>
+        <v>0.44125393140429159</v>
       </c>
       <c r="R33" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A33, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11545,7 +11544,7 @@
       </c>
       <c r="W33" s="25">
         <f t="shared" si="11"/>
-        <v>9.7886318777315644</v>
+        <v>9.7850280865264239</v>
       </c>
       <c r="X33">
         <f t="shared" si="22"/>
@@ -11586,7 +11585,7 @@
       </c>
       <c r="I34" s="44">
         <f t="shared" si="23"/>
-        <v>3.4553535881174102E-2</v>
+        <v>3.4400006643949474E-2</v>
       </c>
       <c r="J34" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A34, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11618,7 +11617,7 @@
       </c>
       <c r="Q34" s="44">
         <f t="shared" si="24"/>
-        <v>0.12557078979625633</v>
+        <v>0.12556624463902757</v>
       </c>
       <c r="R34" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A34, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11638,7 +11637,7 @@
       </c>
       <c r="W34" s="25">
         <f t="shared" si="11"/>
-        <v>5.4652596428169637</v>
+        <v>5.4651015684225106</v>
       </c>
       <c r="X34">
         <f t="shared" si="22"/>
@@ -11679,7 +11678,7 @@
       </c>
       <c r="I35" s="44">
         <f t="shared" si="23"/>
-        <v>0.55985035885591528</v>
+        <v>0.55736281608024485</v>
       </c>
       <c r="J35" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A35, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11711,7 +11710,7 @@
       </c>
       <c r="Q35" s="44">
         <f t="shared" si="24"/>
-        <v>0.2485651855233271</v>
+        <v>0.24855618846396613</v>
       </c>
       <c r="R35" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A35, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11731,7 +11730,7 @@
       </c>
       <c r="W35" s="25">
         <f t="shared" si="11"/>
-        <v>9.6970151777649978</v>
+        <v>9.6945186379299653</v>
       </c>
       <c r="X35">
         <f t="shared" si="22"/>
@@ -11772,7 +11771,7 @@
       </c>
       <c r="I36" s="44">
         <f t="shared" si="23"/>
-        <v>5.5665866375106905E-2</v>
+        <v>5.5418530240437268E-2</v>
       </c>
       <c r="J36" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A36, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11804,7 +11803,7 @@
       </c>
       <c r="Q36" s="44">
         <f t="shared" si="24"/>
-        <v>3.3806301972285131E-2</v>
+        <v>3.3805078320207793E-2</v>
       </c>
       <c r="R36" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A36, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11824,7 +11823,7 @@
       </c>
       <c r="W36" s="25">
         <f t="shared" si="11"/>
-        <v>7.4202539035623651</v>
+        <v>7.4200053437756193</v>
       </c>
       <c r="X36">
         <f t="shared" si="22"/>
@@ -11865,7 +11864,7 @@
       </c>
       <c r="I37" s="44">
         <f t="shared" si="23"/>
-        <v>0.24311927979983733</v>
+        <v>0.24203904541483456</v>
       </c>
       <c r="J37" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A37, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11897,7 +11896,7 @@
       </c>
       <c r="Q37" s="44">
         <f t="shared" si="24"/>
-        <v>0.12589188625218822</v>
+        <v>0.12588732947256004</v>
       </c>
       <c r="R37" s="38">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A37, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11917,7 +11916,7 @@
       </c>
       <c r="W37" s="25">
         <f t="shared" si="11"/>
-        <v>9.1754196313397056</v>
+        <v>9.1743348401750762</v>
       </c>
       <c r="X37">
         <f t="shared" si="22"/>
@@ -11958,7 +11957,7 @@
       </c>
       <c r="I38" s="87">
         <f t="shared" si="23"/>
-        <v>0.17276172524005942</v>
+        <v>0.17199410550965238</v>
       </c>
       <c r="J38" s="86">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A38, Steelhead!$A$3:$A$31, Steelhead!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -11990,7 +11989,7 @@
       </c>
       <c r="Q38" s="87">
         <f t="shared" si="24"/>
-        <v>6.6649469819579671E-2</v>
+        <v>6.6647057377004187E-2</v>
       </c>
       <c r="R38" s="86">
         <f>_xlfn.XLOOKUP(_xlfn.XLOOKUP($A38, 'Bull Trout'!$A$3:$A$31, 'Bull Trout'!$C$3:$C$31),$A$47:$A$51,$B$47:$B$51)</f>
@@ -12010,7 +12009,7 @@
       </c>
       <c r="W38" s="25">
         <f t="shared" si="11"/>
-        <v>11.063774717334283</v>
+        <v>11.0630046851613</v>
       </c>
       <c r="X38">
         <f t="shared" si="22"/>
@@ -12059,11 +12058,11 @@
       </c>
       <c r="H40" s="23">
         <f t="shared" si="25"/>
-        <v>3.7243173501981262</v>
+        <v>3.7409391958819538</v>
       </c>
       <c r="I40" s="85">
         <f t="shared" si="25"/>
-        <v>13.333333333333332</v>
+        <v>13.333333333333336</v>
       </c>
       <c r="J40" s="23">
         <f t="shared" si="25"/>
@@ -12091,11 +12090,11 @@
       </c>
       <c r="P40" s="23">
         <f t="shared" si="25"/>
-        <v>4.2050485144201142</v>
+        <v>4.2052007257624817</v>
       </c>
       <c r="Q40" s="85">
         <f t="shared" si="25"/>
-        <v>13.33333333333333</v>
+        <v>13.333333333333334</v>
       </c>
       <c r="R40" s="23">
         <f t="shared" si="25"/>
@@ -12254,8 +12253,8 @@
         <v>1</v>
       </c>
       <c r="F48" s="46">
-        <f>D16</f>
-        <v>-0.1100000000000001</v>
+        <f>F16</f>
+        <v>0.33333333333333337</v>
       </c>
       <c r="G48" s="47">
         <f>L16</f>
@@ -12281,8 +12280,8 @@
         <v>2</v>
       </c>
       <c r="F49" s="46">
-        <f>F16</f>
-        <v>0.33333333333333337</v>
+        <f>D16</f>
+        <v>-0.1100000000000001</v>
       </c>
       <c r="G49" s="46">
         <f>N16</f>
@@ -12362,8 +12361,8 @@
         <v>1</v>
       </c>
       <c r="F55" s="46">
-        <f>D43</f>
-        <v>0.19974999999999998</v>
+        <f>F43</f>
+        <v>0.34974999999999989</v>
       </c>
       <c r="G55" s="47">
         <f>L43</f>
@@ -12383,8 +12382,8 @@
         <v>2</v>
       </c>
       <c r="F56" s="46">
-        <f>F43</f>
-        <v>0.34974999999999989</v>
+        <f>D43</f>
+        <v>0.19974999999999998</v>
       </c>
       <c r="G56" s="46">
         <f>N43</f>
@@ -12906,7 +12905,7 @@
       <c r="J19" s="2"/>
       <c r="K19" s="1">
         <f>VLOOKUP(A19,'Migration Score Calcs'!$B$1:$F$30,4, FALSE)</f>
-        <v>0</v>
+        <v>1.6621845683827744E-2</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -13964,7 +13963,7 @@
       <c r="K19" s="2"/>
       <c r="L19" s="34">
         <f>VLOOKUP(A19,'Migration Score Calcs'!$B$1:$F$30,5, FALSE)</f>
-        <v>0</v>
+        <v>1.5221134236744052E-4</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
@@ -15566,18 +15565,18 @@
         <v>18</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>3.8577819999999998</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>0.12435499999999999</v>
       </c>
       <c r="E18" s="25">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.6621845683827744E-2</v>
       </c>
       <c r="F18" s="25">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.5221134236744052E-4</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -15866,6 +15865,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FF9AAEF4D584AA4A9EA65E175D94333C" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="19e2b9843ca88f851965d64f9b369b1b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d05db09f-8a2c-4258-8a75-47a1515983ff" xmlns:ns3="43ccd64e-69b8-4e29-9547-c09289680468" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="08418edd0ca35abc814edd24e7526acc" ns2:_="" ns3:_="">
     <xsd:import namespace="d05db09f-8a2c-4258-8a75-47a1515983ff"/>
@@ -16072,33 +16080,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75A1F728-59E6-44B1-B183-30105A117FDE}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="43ccd64e-69b8-4e29-9547-c09289680468"/>
+    <ds:schemaRef ds:uri="d05db09f-8a2c-4258-8a75-47a1515983ff"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="43ccd64e-69b8-4e29-9547-c09289680468"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="d05db09f-8a2c-4258-8a75-47a1515983ff"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD943BF4-FA33-4111-B18F-FFEF53A64004}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B6D3807-8F2B-4D6E-AB26-DF9064F0C4B6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -16115,12 +16122,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD943BF4-FA33-4111-B18F-FFEF53A64004}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>